<commit_message>
EOD 2026-07-22: ZERO tradeable names. Full universe 155/156 on candles; 29 fresh Chandelier BUY signals culled to 0 by the regime+ADX+DI+ZLSMA stack (last survivor SKK killed on 84.5k dollar ADV). Yesterday's calls scored: gates-passed +1.19 pct vs gates-blocked -1.12 pct, fresh beat stale by 2.7 pts, SPY flat. 76 of 155 names in sell mode, all five index/sector proxies in sell mode. Adds EOD brief + universe workbook in the new layout + build_universe_results.py bridge.
</commit_message>
<xml_diff>
--- a/reports/plans_2026-07-21.xlsx
+++ b/reports/plans_2026-07-21.xlsx
@@ -21,13 +21,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
@@ -63,13 +67,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -452,189 +457,196 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Entry (limit)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Size</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Risk $</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Targets</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Earnings gate</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Status / Notes</t>
+          <t>Plan data as of Mon 2026-07-20 close + Tue 7/21 AM decisions · written 2026-07-21 13:52 local</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Entry (limit)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Risk $</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Targets</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Earnings gate</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Status / Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>BHP</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>BHP Group ADR (mining) — NYSE listing, USD; ASX shows ~AUD 58 = same value</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C3" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D3" s="3" t="n">
         <v>76.59999999999999</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>half $50k (~625sh)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F3" s="3" t="n">
         <v>2100</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>86.30 then 88</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>FY results 8/17-18 (clear runway)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Alert 5195389330 armed. Fresh 7/15 buy, regime PASS +13.7% over 200d; record FY26 iron ore + ~2Mt copper already reported</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>ECVT</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Ecovyst (specialty chemicals)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>12.35</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D4" s="3" t="n">
         <v>11.55</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>half $40k (~3,240sh)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <v>2600</v>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>13.07 then 14</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>8/5 BMO — trim 8/4</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Alert 5195389391 armed. Fresh 7/16-17 base breakout, regime PASS, ADX 29 — cleanest new chart of the run</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>NUE</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Nucor (steel)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Q2 7/27 AMC</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Omar passed 7/21 AM — graded as SKIP vs ref 231.00. Stop alert 5189401855 now informational</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>PFE</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Pfizer (pharma)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>8/4 BMO + PDUFA 8/17</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Omar passed 7/21 AM — graded as SKIP vs ref 24.86. Stop alert 5189401903 now informational</t>
         </is>
@@ -651,7 +663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -666,132 +678,139 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Trigger level</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Then</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Earnings</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
+          <t>Plan data as of Mon 2026-07-20 close + Tue 7/21 AM decisions · written 2026-07-21 13:52 local</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Trigger level</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Then</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>GS</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Goldman Sachs</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C3" s="3" t="n">
         <v>1078</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>BUY half $50k (~46sh)</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E3" s="3" t="n">
         <v>1025</v>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>behind (Q2 beat 7/14); next ~10/14</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Alert 5195389473. Fresh 7/15, regime PASS; blocked only by being under ZLSMA — buy the reclaim, target 1,154 then 1,190</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>MAC</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Macerich (mall REIT)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>26.2</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>BUY starter $25k (~950sh)</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <v>24.4</v>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>8/4 AMC — trim 8/3</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Alert 5195389644. Mall-REIT cluster: MAC+SPG+M all fresh 7/16-17; MAC = gated vehicle; target 28</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>TLN</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Talen Energy (power)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C5" s="3" t="n">
         <v>389</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>starter only, re-run gates first</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>8/5 AMC</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Alert 5195389568. PJM $1.21B capacity catalyst confirmed, but under ZLSMA + regime REPAIR — reclaim first</t>
         </is>
@@ -808,7 +827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -820,108 +839,115 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>When</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>What to do</t>
+          <t>Plan data as of Mon 2026-07-20 close + Tue 7/21 AM decisions · written 2026-07-21 13:52 local</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>HAS</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Q2 earnings</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Tue 7/21 BMO (this morning)</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Fresh 7/16 buy went into the print — check the reaction; clean print = the benched signal re-opens</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>COCO</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Q2 earnings</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Thu 7/23 BMO</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Best regime score of the whole scan (+29.2% over 200d) — re-look after the print, do NOT enter before</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>VZ</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Q2 earnings</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Fri 7/24 BMO</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Fresh Fri 7/17 signal but zero runway — decide after the print</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>CEG</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>OMAR DECISION PENDING</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>now</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Live 245 buy alert vs regime DEEP-FAIL (−18.9% below 200d; frozen rules say watch-only). Keep or pull?</t>
         </is>
@@ -938,7 +964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -948,226 +974,233 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Reason</t>
+          <t>Plan data as of Mon 2026-07-20 close + Tue 7/21 AM decisions · written 2026-07-21 13:52 local</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>ODFL</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Magical +115 too hot; trucking pair with XPO — XPO (208 alert) is the vehicle</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>SPG</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Magical +118 too hot; mall-REIT cluster — MAC is the vehicle</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>LCID</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Dead-cat: buy printed right after a crash candle, Magical +152</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>NOV</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Magical +149 + regime REPAIR (oil-services V-bottom)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>WPC</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Magical +187 — vertical 5-bar rally</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>BG</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Magical +137 (V-bottom)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>CHRD</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Magical +146 (V-bottom)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>HLX</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Magical +103; oil-services theme with NOV</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>RYZ</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Magical +125 AND listing ambiguity (Ryerson normally trades RYI) — verify before ever acting</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>CVNA</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Regime deep-fail: −11.8% below 200d, RS −37 vs SPY</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>SHAK</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Regime deep-fail: −31.7% below 200d</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>VVV</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Under ZLSMA — watch a ~40.50 reclaim; earnings 8/5</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Under ZLSMA + whipsaw (sell flip only ~10 bars prior); mall-retail cluster member</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>FNB</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Re-flipped to buy ONE day after a sell flip — classic CE(1,2) chop</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>FLG</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Under ZLSMA, negative Magical — likely whipsaw</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>TRNS</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Whipsaw + red candles since signal + thin volume</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>CNOB</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Thin (~577K/day) + under ZLSMA</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>SPXL</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>3x ETP — market-read note only (big-caps-ex-tech holding while QQQ/SMH in sell mode)</t>
         </is>
@@ -1184,7 +1217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1198,105 +1231,88 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Plan data as of Mon 2026-07-20 close + Tue 7/21 AM decisions · written 2026-07-21 13:52 local</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>29% of covered July recs broke within 30 days — be picky with fresh signals</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>% since rec</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Rec price</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Last</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Magical</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Reason</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>29% of covered July recs broke within 30 days — be picky with fresh signals</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TTI</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>-19.9</v>
-      </c>
-      <c r="C2" t="n">
-        <v>11.33</v>
-      </c>
-      <c r="D2" t="n">
-        <v>9.07</v>
-      </c>
-      <c r="E2" t="n">
-        <v>-85.3</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>early failure: rec 20d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DSGN</t>
+          <t>TTI</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-17.3</v>
+        <v>-19.9</v>
       </c>
       <c r="C3" t="n">
-        <v>14.85</v>
+        <v>11.33</v>
       </c>
       <c r="D3" t="n">
-        <v>12.28</v>
+        <v>9.07</v>
       </c>
       <c r="E3" t="n">
-        <v>-162.2</v>
+        <v>-85.3</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>early failure: rec 14d ago now sell-mode</t>
+          <t>early failure: rec 20d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ALHC</t>
+          <t>DSGN</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-15.2</v>
+        <v>-17.3</v>
       </c>
       <c r="C4" t="n">
-        <v>24.56</v>
+        <v>14.85</v>
       </c>
       <c r="D4" t="n">
-        <v>20.83</v>
+        <v>12.28</v>
       </c>
       <c r="E4" t="n">
-        <v>-63.1</v>
+        <v>-162.2</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1307,92 +1323,92 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>ALHC</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-13.8</v>
+        <v>-15.2</v>
       </c>
       <c r="C5" t="n">
-        <v>385.95</v>
+        <v>24.56</v>
       </c>
       <c r="D5" t="n">
-        <v>332.7</v>
+        <v>20.83</v>
       </c>
       <c r="E5" t="n">
-        <v>-289.8</v>
+        <v>-63.1</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>early failure: rec 11d ago now sell-mode</t>
+          <t>early failure: rec 14d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>WRBY</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-12.6</v>
+        <v>-13.8</v>
       </c>
       <c r="C6" t="n">
-        <v>29.22</v>
+        <v>385.95</v>
       </c>
       <c r="D6" t="n">
-        <v>25.53</v>
+        <v>332.7</v>
       </c>
       <c r="E6" t="n">
-        <v>-141.1</v>
+        <v>-289.8</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>early failure: rec 14d ago now sell-mode</t>
+          <t>early failure: rec 11d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SSD</t>
+          <t>WRBY</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-10.4</v>
+        <v>-12.6</v>
       </c>
       <c r="C7" t="n">
-        <v>209.35</v>
+        <v>29.22</v>
       </c>
       <c r="D7" t="n">
-        <v>187.65</v>
+        <v>25.53</v>
       </c>
       <c r="E7" t="n">
-        <v>-85.3</v>
+        <v>-141.1</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>early failure: rec 20d ago now sell-mode</t>
+          <t>early failure: rec 14d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NPKI</t>
+          <t>SSD</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-9.4</v>
+        <v>-10.4</v>
       </c>
       <c r="C8" t="n">
-        <v>15.91</v>
+        <v>209.35</v>
       </c>
       <c r="D8" t="n">
-        <v>14.41</v>
+        <v>187.65</v>
       </c>
       <c r="E8" t="n">
-        <v>-42.9</v>
+        <v>-85.3</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1403,284 +1419,284 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>KURA</t>
+          <t>NPKI</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-9.300000000000001</v>
+        <v>-9.4</v>
       </c>
       <c r="C9" t="n">
-        <v>11.99</v>
+        <v>15.91</v>
       </c>
       <c r="D9" t="n">
-        <v>10.88</v>
+        <v>14.41</v>
       </c>
       <c r="E9" t="n">
-        <v>-28.2</v>
+        <v>-42.9</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>early failure: rec 13d ago now sell-mode</t>
+          <t>early failure: rec 20d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AROC</t>
+          <t>KURA</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-8.5</v>
+        <v>-9.300000000000001</v>
       </c>
       <c r="C10" t="n">
-        <v>40.71</v>
+        <v>11.99</v>
       </c>
       <c r="D10" t="n">
-        <v>37.23</v>
+        <v>10.88</v>
       </c>
       <c r="E10" t="n">
-        <v>-82.8</v>
+        <v>-28.2</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>early failure: rec 20d ago now sell-mode</t>
+          <t>early failure: rec 13d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BIOA</t>
+          <t>AROC</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-8.199999999999999</v>
+        <v>-8.5</v>
       </c>
       <c r="C11" t="n">
-        <v>24.84</v>
+        <v>40.71</v>
       </c>
       <c r="D11" t="n">
-        <v>22.8</v>
+        <v>37.23</v>
       </c>
       <c r="E11" t="n">
-        <v>-35.4</v>
+        <v>-82.8</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>early failure: rec 14d ago now sell-mode</t>
+          <t>early failure: rec 20d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>BIOA</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-8</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="C12" t="n">
-        <v>140.79</v>
+        <v>24.84</v>
       </c>
       <c r="D12" t="n">
-        <v>129.5</v>
+        <v>22.8</v>
       </c>
       <c r="E12" t="n">
-        <v>-182.5</v>
+        <v>-35.4</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>early failure: rec 11d ago now sell-mode</t>
+          <t>early failure: rec 14d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MAMA</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="C13" t="n">
-        <v>18.33</v>
+        <v>140.79</v>
       </c>
       <c r="D13" t="n">
-        <v>17.04</v>
+        <v>129.5</v>
       </c>
       <c r="E13" t="n">
-        <v>-168</v>
+        <v>-182.5</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>early failure: rec 19d ago now sell-mode</t>
+          <t>early failure: rec 11d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OSCR</t>
+          <t>MAMA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-6.7</v>
+        <v>-7</v>
       </c>
       <c r="C14" t="n">
-        <v>31.44</v>
+        <v>18.33</v>
       </c>
       <c r="D14" t="n">
-        <v>29.33</v>
+        <v>17.04</v>
       </c>
       <c r="E14" t="n">
-        <v>-56.2</v>
+        <v>-168</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>early failure: rec 14d ago now sell-mode</t>
+          <t>early failure: rec 19d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>OSCR</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-6.5</v>
+        <v>-6.7</v>
       </c>
       <c r="C15" t="n">
-        <v>546.72</v>
+        <v>31.44</v>
       </c>
       <c r="D15" t="n">
-        <v>511.34</v>
+        <v>29.33</v>
       </c>
       <c r="E15" t="n">
-        <v>-73.09999999999999</v>
+        <v>-56.2</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>early failure: rec 11d ago now sell-mode</t>
+          <t>early failure: rec 14d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-6.3</v>
+        <v>-6.5</v>
       </c>
       <c r="C16" t="n">
-        <v>320.42</v>
+        <v>546.72</v>
       </c>
       <c r="D16" t="n">
-        <v>300.08</v>
+        <v>511.34</v>
       </c>
       <c r="E16" t="n">
-        <v>-16.2</v>
+        <v>-73.09999999999999</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>early failure: rec 14d ago now sell-mode</t>
+          <t>early failure: rec 11d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SENEA</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>-6.3</v>
       </c>
       <c r="C17" t="n">
-        <v>177.76</v>
+        <v>320.42</v>
       </c>
       <c r="D17" t="n">
-        <v>166.51</v>
+        <v>300.08</v>
       </c>
       <c r="E17" t="n">
-        <v>-59.2</v>
+        <v>-16.2</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>early failure: rec 12d ago now sell-mode</t>
+          <t>early failure: rec 14d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>SENEA</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-6.2</v>
+        <v>-6.3</v>
       </c>
       <c r="C18" t="n">
-        <v>417.28</v>
+        <v>177.76</v>
       </c>
       <c r="D18" t="n">
-        <v>391.6</v>
+        <v>166.51</v>
       </c>
       <c r="E18" t="n">
-        <v>-110.3</v>
+        <v>-59.2</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>early failure: rec 13d ago now sell-mode</t>
+          <t>early failure: rec 12d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>OPY</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-6.1</v>
+        <v>-6.2</v>
       </c>
       <c r="C19" t="n">
-        <v>115.47</v>
+        <v>417.28</v>
       </c>
       <c r="D19" t="n">
-        <v>108.37</v>
+        <v>391.6</v>
       </c>
       <c r="E19" t="n">
-        <v>-52</v>
+        <v>-110.3</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>early failure: rec 14d ago now sell-mode</t>
+          <t>early failure: rec 13d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BSTZ</t>
+          <t>OPY</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-5.9</v>
+        <v>-6.1</v>
       </c>
       <c r="C20" t="n">
-        <v>29.62</v>
+        <v>115.47</v>
       </c>
       <c r="D20" t="n">
-        <v>27.86</v>
+        <v>108.37</v>
       </c>
       <c r="E20" t="n">
-        <v>-138.5</v>
+        <v>-52</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1691,140 +1707,140 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PTCT</t>
+          <t>BSTZ</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-5.8</v>
+        <v>-5.9</v>
       </c>
       <c r="C21" t="n">
-        <v>83.31</v>
+        <v>29.62</v>
       </c>
       <c r="D21" t="n">
-        <v>78.48</v>
+        <v>27.86</v>
       </c>
       <c r="E21" t="n">
-        <v>-104.7</v>
+        <v>-138.5</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>early failure: rec 19d ago now sell-mode</t>
+          <t>early failure: rec 14d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BFC</t>
+          <t>PTCT</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>-5.8</v>
       </c>
       <c r="C22" t="n">
-        <v>153.21</v>
+        <v>83.31</v>
       </c>
       <c r="D22" t="n">
-        <v>144.3</v>
+        <v>78.48</v>
       </c>
       <c r="E22" t="n">
-        <v>-101.7</v>
+        <v>-104.7</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>early failure: rec 4d ago now sell-mode</t>
+          <t>early failure: rec 19d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FCFS</t>
+          <t>BFC</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-5.5</v>
+        <v>-5.8</v>
       </c>
       <c r="C23" t="n">
-        <v>224.29</v>
+        <v>153.21</v>
       </c>
       <c r="D23" t="n">
-        <v>212.02</v>
+        <v>144.3</v>
       </c>
       <c r="E23" t="n">
-        <v>-110.4</v>
+        <v>-101.7</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>early failure: rec 14d ago now sell-mode</t>
+          <t>early failure: rec 4d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>FCFS</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-5</v>
+        <v>-5.5</v>
       </c>
       <c r="C24" t="n">
-        <v>28.57</v>
+        <v>224.29</v>
       </c>
       <c r="D24" t="n">
-        <v>27.14</v>
+        <v>212.02</v>
       </c>
       <c r="E24" t="n">
-        <v>-50.5</v>
+        <v>-110.4</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>early failure: rec 19d ago now sell-mode</t>
+          <t>early failure: rec 14d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ALKS</t>
+          <t>EGBN</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>-5</v>
       </c>
       <c r="C25" t="n">
-        <v>55.14</v>
+        <v>28.57</v>
       </c>
       <c r="D25" t="n">
-        <v>52.41</v>
+        <v>27.14</v>
       </c>
       <c r="E25" t="n">
-        <v>14.9</v>
+        <v>-50.5</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>early failure: rec 14d ago now sell-mode</t>
+          <t>early failure: rec 19d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>ALKS</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>-4.5</v>
+        <v>-5</v>
       </c>
       <c r="C26" t="n">
-        <v>79.06999999999999</v>
+        <v>55.14</v>
       </c>
       <c r="D26" t="n">
-        <v>75.54000000000001</v>
+        <v>52.41</v>
       </c>
       <c r="E26" t="n">
-        <v>0.9</v>
+        <v>14.9</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1835,20 +1851,20 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CACC</t>
+          <t>FTDR</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>-4.4</v>
+        <v>-4.5</v>
       </c>
       <c r="C27" t="n">
-        <v>657.2</v>
+        <v>79.06999999999999</v>
       </c>
       <c r="D27" t="n">
-        <v>628.3099999999999</v>
+        <v>75.54000000000001</v>
       </c>
       <c r="E27" t="n">
-        <v>7.3</v>
+        <v>0.9</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1859,20 +1875,20 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>NWPX</t>
+          <t>CACC</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>-3.7</v>
+        <v>-4.4</v>
       </c>
       <c r="C28" t="n">
-        <v>143.18</v>
+        <v>657.2</v>
       </c>
       <c r="D28" t="n">
-        <v>137.85</v>
+        <v>628.3099999999999</v>
       </c>
       <c r="E28" t="n">
-        <v>-29.8</v>
+        <v>7.3</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1883,20 +1899,20 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>NWPX</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>-3.4</v>
+        <v>-3.7</v>
       </c>
       <c r="C29" t="n">
-        <v>487.24</v>
+        <v>143.18</v>
       </c>
       <c r="D29" t="n">
-        <v>470.75</v>
+        <v>137.85</v>
       </c>
       <c r="E29" t="n">
-        <v>-113.7</v>
+        <v>-29.8</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1907,20 +1923,20 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CPT</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>-3.3</v>
+        <v>-3.4</v>
       </c>
       <c r="C30" t="n">
-        <v>116.95</v>
+        <v>487.24</v>
       </c>
       <c r="D30" t="n">
-        <v>113.1</v>
+        <v>470.75</v>
       </c>
       <c r="E30" t="n">
-        <v>-34.7</v>
+        <v>-113.7</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1931,20 +1947,20 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>EXTR</t>
+          <t>CPT</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>-3.3</v>
       </c>
       <c r="C31" t="n">
-        <v>31.33</v>
+        <v>116.95</v>
       </c>
       <c r="D31" t="n">
-        <v>30.31</v>
+        <v>113.1</v>
       </c>
       <c r="E31" t="n">
-        <v>-81.2</v>
+        <v>-34.7</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1955,20 +1971,20 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>LEVI</t>
+          <t>EXTR</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>-2.7</v>
+        <v>-3.3</v>
       </c>
       <c r="C32" t="n">
-        <v>24.68</v>
+        <v>31.33</v>
       </c>
       <c r="D32" t="n">
-        <v>24.02</v>
+        <v>30.31</v>
       </c>
       <c r="E32" t="n">
-        <v>-29.1</v>
+        <v>-81.2</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1979,116 +1995,116 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IBKR</t>
+          <t>LEVI</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>-2.7</v>
       </c>
       <c r="C33" t="n">
-        <v>94.56999999999999</v>
+        <v>24.68</v>
       </c>
       <c r="D33" t="n">
-        <v>92</v>
+        <v>24.02</v>
       </c>
       <c r="E33" t="n">
-        <v>-41.4</v>
+        <v>-29.1</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>early failure: rec 13d ago now sell-mode</t>
+          <t>early failure: rec 14d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>IBKR</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>-2.1</v>
+        <v>-2.7</v>
       </c>
       <c r="C34" t="n">
-        <v>74.73</v>
+        <v>94.56999999999999</v>
       </c>
       <c r="D34" t="n">
-        <v>73.16</v>
+        <v>92</v>
       </c>
       <c r="E34" t="n">
-        <v>56.5</v>
+        <v>-41.4</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>early failure: rec 4d ago now sell-mode</t>
+          <t>early failure: rec 13d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SRRK</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>-2</v>
+        <v>-2.1</v>
       </c>
       <c r="C35" t="n">
-        <v>52.84</v>
+        <v>74.73</v>
       </c>
       <c r="D35" t="n">
-        <v>51.77</v>
+        <v>73.16</v>
       </c>
       <c r="E35" t="n">
-        <v>-80.2</v>
+        <v>56.5</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>early failure: rec 19d ago now sell-mode</t>
+          <t>early failure: rec 4d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>SRRK</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>-2</v>
       </c>
       <c r="C36" t="n">
-        <v>173.28</v>
+        <v>52.84</v>
       </c>
       <c r="D36" t="n">
-        <v>169.8</v>
+        <v>51.77</v>
       </c>
       <c r="E36" t="n">
-        <v>-4</v>
+        <v>-80.2</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>early failure: rec 14d ago now sell-mode</t>
+          <t>early failure: rec 19d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>-1.3</v>
+        <v>-2</v>
       </c>
       <c r="C37" t="n">
-        <v>419.03</v>
+        <v>173.28</v>
       </c>
       <c r="D37" t="n">
-        <v>413.43</v>
+        <v>169.8</v>
       </c>
       <c r="E37" t="n">
-        <v>17.6</v>
+        <v>-4</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2099,190 +2115,214 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>FFIV</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>-1.3</v>
       </c>
       <c r="C38" t="n">
-        <v>127.63</v>
+        <v>419.03</v>
       </c>
       <c r="D38" t="n">
-        <v>125.95</v>
+        <v>413.43</v>
       </c>
       <c r="E38" t="n">
-        <v>21.6</v>
+        <v>17.6</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>early failure: rec 4d ago now sell-mode</t>
+          <t>early failure: rec 14d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SJM</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>-0.8</v>
+        <v>-1.3</v>
       </c>
       <c r="C39" t="n">
-        <v>113.24</v>
+        <v>127.63</v>
       </c>
       <c r="D39" t="n">
-        <v>112.37</v>
+        <v>125.95</v>
       </c>
       <c r="E39" t="n">
-        <v>-1</v>
+        <v>21.6</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>early failure: rec 13d ago now sell-mode</t>
+          <t>early failure: rec 4d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>SJM</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>-0.7</v>
+        <v>-0.8</v>
       </c>
       <c r="C40" t="n">
-        <v>29.3</v>
+        <v>113.24</v>
       </c>
       <c r="D40" t="n">
-        <v>29.1</v>
+        <v>112.37</v>
       </c>
       <c r="E40" t="n">
-        <v>-27</v>
+        <v>-1</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>early failure: rec 20d ago now sell-mode</t>
+          <t>early failure: rec 13d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>LSTR</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>-0.6</v>
+        <v>-0.7</v>
       </c>
       <c r="C41" t="n">
-        <v>212.87</v>
+        <v>29.3</v>
       </c>
       <c r="D41" t="n">
-        <v>211.61</v>
+        <v>29.1</v>
       </c>
       <c r="E41" t="n">
-        <v>99.3</v>
+        <v>-27</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>early failure: rec 8d ago now sell-mode</t>
+          <t>early failure: rec 20d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SLAB</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>-0.4</v>
+        <v>-0.6</v>
       </c>
       <c r="C42" t="n">
-        <v>218.37</v>
+        <v>212.87</v>
       </c>
       <c r="D42" t="n">
-        <v>217.57</v>
+        <v>211.61</v>
       </c>
       <c r="E42" t="n">
-        <v>-128.9</v>
+        <v>99.3</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>early failure: rec 4d ago now sell-mode</t>
+          <t>early failure: rec 8d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>LYV</t>
+          <t>SLAB</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>-0.3</v>
+        <v>-0.4</v>
       </c>
       <c r="C43" t="n">
-        <v>182.14</v>
+        <v>218.37</v>
       </c>
       <c r="D43" t="n">
-        <v>181.61</v>
+        <v>217.57</v>
       </c>
       <c r="E43" t="n">
-        <v>32.7</v>
+        <v>-128.9</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>early failure: rec 12d ago now sell-mode</t>
+          <t>early failure: rec 4d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>LYV</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.1</v>
+        <v>-0.3</v>
       </c>
       <c r="C44" t="n">
-        <v>352.16</v>
+        <v>182.14</v>
       </c>
       <c r="D44" t="n">
-        <v>352.51</v>
+        <v>181.61</v>
       </c>
       <c r="E44" t="n">
-        <v>56.7</v>
+        <v>32.7</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>early failure: rec 4d ago now sell-mode</t>
+          <t>early failure: rec 12d ago now sell-mode</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>352.16</v>
+      </c>
+      <c r="D45" t="n">
+        <v>352.51</v>
+      </c>
+      <c r="E45" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>early failure: rec 4d ago now sell-mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>ASB</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B46" t="n">
         <v>1.8</v>
       </c>
-      <c r="C45" t="n">
+      <c r="C46" t="n">
         <v>30.6</v>
       </c>
-      <c r="D45" t="n">
+      <c r="D46" t="n">
         <v>31.16</v>
       </c>
-      <c r="E45" t="n">
+      <c r="E46" t="n">
         <v>83.7</v>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>early failure: rec 11d ago now sell-mode</t>
         </is>

</xml_diff>